<commit_message>
Amelioration de  ML (MODÈLE DE COÛT)
</commit_message>
<xml_diff>
--- a/backend/data/data.xlsx
+++ b/backend/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Stage_Day_Machines\repair-platform\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4BE5EBC-B6A6-4983-94FD-DE5CCA8F237C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA86442F-4B0A-4240-81A9-F5F5B0C17BE0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{7BC39F58-AA9C-4CC8-9008-01B13AEFA6DB}"/>
   </bookViews>
@@ -542,7 +542,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="[$-40C]dd\-mmm\-yy"/>
+    <numFmt numFmtId="164" formatCode="[$-40C]dd\-mmm\-yy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -628,7 +628,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
@@ -5914,7 +5914,7 @@
         <v>149</v>
       </c>
       <c r="I131">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J131" t="s">
         <v>58</v>
@@ -5952,7 +5952,7 @@
         <v>149</v>
       </c>
       <c r="I132">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J132" t="s">
         <v>58</v>
@@ -5990,7 +5990,7 @@
         <v>149</v>
       </c>
       <c r="I133">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J133" t="s">
         <v>58</v>
@@ -8080,7 +8080,7 @@
         <v>151</v>
       </c>
       <c r="I188">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J188" t="s">
         <v>58</v>
@@ -10930,7 +10930,7 @@
         <v>149</v>
       </c>
       <c r="I263" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J263" t="s">
         <v>58</v>
@@ -10968,7 +10968,7 @@
         <v>149</v>
       </c>
       <c r="I264" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J264" t="s">
         <v>58</v>
@@ -11006,7 +11006,7 @@
         <v>149</v>
       </c>
       <c r="I265">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J265" t="s">
         <v>58</v>
@@ -12222,7 +12222,7 @@
         <v>149</v>
       </c>
       <c r="I297">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J297" t="s">
         <v>58</v>
@@ -12374,7 +12374,7 @@
         <v>133</v>
       </c>
       <c r="I301">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J301" t="s">
         <v>58</v>
@@ -12640,7 +12640,7 @@
         <v>149</v>
       </c>
       <c r="I308">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J308" t="s">
         <v>58</v>
@@ -12678,7 +12678,7 @@
         <v>149</v>
       </c>
       <c r="I309">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="J309" t="s">
         <v>58</v>
@@ -12868,7 +12868,7 @@
         <v>151</v>
       </c>
       <c r="I314">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J314" t="s">
         <v>58</v>
@@ -13210,7 +13210,7 @@
         <v>149</v>
       </c>
       <c r="I323">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J323" t="s">
         <v>58</v>
@@ -13248,7 +13248,7 @@
         <v>133</v>
       </c>
       <c r="I324">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J324" t="s">
         <v>58</v>
@@ -13552,7 +13552,7 @@
         <v>133</v>
       </c>
       <c r="I332">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J332" t="s">
         <v>58</v>
@@ -14464,7 +14464,7 @@
         <v>133</v>
       </c>
       <c r="I356">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="J356" t="s">
         <v>58</v>
@@ -14616,7 +14616,7 @@
         <v>133</v>
       </c>
       <c r="I360">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="J360" t="s">
         <v>58</v>
@@ -14768,7 +14768,7 @@
         <v>149</v>
       </c>
       <c r="I364">
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="J364" t="s">
         <v>58</v>
@@ -15452,7 +15452,7 @@
         <v>149</v>
       </c>
       <c r="I382" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J382" t="s">
         <v>58</v>
@@ -15490,7 +15490,7 @@
         <v>149</v>
       </c>
       <c r="I383" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J383" t="s">
         <v>58</v>
@@ -15528,7 +15528,7 @@
         <v>149</v>
       </c>
       <c r="I384">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J384" t="s">
         <v>58</v>
@@ -16858,7 +16858,7 @@
         <v>149</v>
       </c>
       <c r="I419">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J419" t="s">
         <v>58</v>
@@ -17010,7 +17010,7 @@
         <v>133</v>
       </c>
       <c r="I423">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J423" t="s">
         <v>58</v>
@@ -17276,7 +17276,7 @@
         <v>149</v>
       </c>
       <c r="I430">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J430" t="s">
         <v>58</v>
@@ -17314,7 +17314,7 @@
         <v>149</v>
       </c>
       <c r="I431">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="J431" t="s">
         <v>58</v>
@@ -17504,7 +17504,7 @@
         <v>151</v>
       </c>
       <c r="I436">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J436" t="s">
         <v>58</v>
@@ -17808,7 +17808,7 @@
         <v>149</v>
       </c>
       <c r="I444">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J444" t="s">
         <v>58</v>
@@ -17846,7 +17846,7 @@
         <v>133</v>
       </c>
       <c r="I445">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J445" t="s">
         <v>58</v>
@@ -18188,7 +18188,7 @@
         <v>133</v>
       </c>
       <c r="I454">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J454" t="s">
         <v>58</v>
@@ -19100,7 +19100,7 @@
         <v>133</v>
       </c>
       <c r="I478">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="J478" t="s">
         <v>58</v>
@@ -19214,7 +19214,7 @@
         <v>133</v>
       </c>
       <c r="I481">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="J481" t="s">
         <v>58</v>
@@ -19366,7 +19366,7 @@
         <v>149</v>
       </c>
       <c r="I485">
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="J485" t="s">
         <v>58</v>
@@ -20164,7 +20164,7 @@
         <v>149</v>
       </c>
       <c r="I506">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J506" t="s">
         <v>58</v>
@@ -20240,7 +20240,7 @@
         <v>149</v>
       </c>
       <c r="I508">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J508" t="s">
         <v>58</v>
@@ -21532,7 +21532,7 @@
         <v>149</v>
       </c>
       <c r="I542">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="J542" t="s">
         <v>58</v>
@@ -21722,7 +21722,7 @@
         <v>133</v>
       </c>
       <c r="I547">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="J547" t="s">
         <v>58</v>
@@ -21988,7 +21988,7 @@
         <v>149</v>
       </c>
       <c r="I554">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J554" t="s">
         <v>58</v>
@@ -22178,7 +22178,7 @@
         <v>151</v>
       </c>
       <c r="I559">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J559" t="s">
         <v>58</v>
@@ -22406,7 +22406,7 @@
         <v>149</v>
       </c>
       <c r="I565">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J565" t="s">
         <v>58</v>
@@ -22520,7 +22520,7 @@
         <v>149</v>
       </c>
       <c r="I568">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J568" t="s">
         <v>58</v>
@@ -22786,7 +22786,7 @@
         <v>151</v>
       </c>
       <c r="I575">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J575" t="s">
         <v>58</v>
@@ -22900,7 +22900,7 @@
         <v>133</v>
       </c>
       <c r="I578" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J578" t="s">
         <v>58</v>
@@ -23812,7 +23812,7 @@
         <v>133</v>
       </c>
       <c r="I602">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J602" t="s">
         <v>58</v>
@@ -23926,7 +23926,7 @@
         <v>133</v>
       </c>
       <c r="I605">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="J605" t="s">
         <v>58</v>
@@ -24116,7 +24116,7 @@
         <v>149</v>
       </c>
       <c r="I610">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J610" t="s">
         <v>58</v>
@@ -24800,7 +24800,7 @@
         <v>149</v>
       </c>
       <c r="I628">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J628" t="s">
         <v>58</v>
@@ -24876,7 +24876,7 @@
         <v>149</v>
       </c>
       <c r="I630">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J630" t="s">
         <v>58</v>
@@ -26092,7 +26092,7 @@
         <v>149</v>
       </c>
       <c r="I662">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="J662" t="s">
         <v>58</v>
@@ -26282,7 +26282,7 @@
         <v>133</v>
       </c>
       <c r="I667">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="J667" t="s">
         <v>58</v>
@@ -26548,7 +26548,7 @@
         <v>149</v>
       </c>
       <c r="I674">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J674" t="s">
         <v>58</v>
@@ -27042,7 +27042,7 @@
         <v>149</v>
       </c>
       <c r="I687">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J687" t="s">
         <v>58</v>
@@ -27270,7 +27270,7 @@
         <v>151</v>
       </c>
       <c r="I693">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J693" t="s">
         <v>58</v>
@@ -27384,7 +27384,7 @@
         <v>133</v>
       </c>
       <c r="I696" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J696" t="s">
         <v>58</v>
@@ -28296,7 +28296,7 @@
         <v>133</v>
       </c>
       <c r="I720">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J720" t="s">
         <v>58</v>
@@ -28410,7 +28410,7 @@
         <v>133</v>
       </c>
       <c r="I723">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="J723" t="s">
         <v>58</v>
@@ -28600,7 +28600,7 @@
         <v>149</v>
       </c>
       <c r="I728">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="J728" t="s">
         <v>58</v>
@@ -29360,7 +29360,7 @@
         <v>149</v>
       </c>
       <c r="I748">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J748" t="s">
         <v>58</v>
@@ -29398,7 +29398,7 @@
         <v>149</v>
       </c>
       <c r="I749">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="J749" t="s">
         <v>58</v>
@@ -29436,7 +29436,7 @@
         <v>149</v>
       </c>
       <c r="I750">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J750" t="s">
         <v>58</v>
@@ -30690,7 +30690,7 @@
         <v>149</v>
       </c>
       <c r="I783">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J783" t="s">
         <v>58</v>
@@ -31108,7 +31108,7 @@
         <v>149</v>
       </c>
       <c r="I794">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J794" t="s">
         <v>58</v>
@@ -31146,7 +31146,7 @@
         <v>149</v>
       </c>
       <c r="I795">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="J795" t="s">
         <v>58</v>
@@ -31564,7 +31564,7 @@
         <v>149</v>
       </c>
       <c r="I806">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="J806" t="s">
         <v>58</v>
@@ -31678,7 +31678,7 @@
         <v>149</v>
       </c>
       <c r="I809">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="J809" t="s">
         <v>58</v>
@@ -31944,7 +31944,7 @@
         <v>151</v>
       </c>
       <c r="I816" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J816" t="s">
         <v>58</v>
@@ -32058,7 +32058,7 @@
         <v>133</v>
       </c>
       <c r="I819">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J819" t="s">
         <v>58</v>
@@ -33160,7 +33160,7 @@
         <v>133</v>
       </c>
       <c r="I848">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="J848" t="s">
         <v>58</v>
@@ -33350,7 +33350,7 @@
         <v>149</v>
       </c>
       <c r="I853">
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="J853" t="s">
         <v>58</v>

</xml_diff>